<commit_message>
Add remove-from-cart test flow and fix flaky waits/popup handling
- Add RemoveProductFromCartTest and RemoveProductsFromCartPAge for the new-UI remove-from-cart flow
- Fix implicit wait bleeding into explicit waits in CommonUtils (clickRetryingPopup, clickIfPresent) so timeouts fail fast instead of stacking up to ~90s
- Disable the encircle-popup auto-retry-everywhere behavior that was causing cascading test retries; keep explicit dismissEncirclePopupIfPresent() calls at known points
- Force app data reset before each session (noReset=false) so login screen shows every run
- Set enforceXPath1 to keep UiAutomator2 on the XPath 1.0 evaluator the app's locators were written against
- Update PurchaseTestNew, CartPageElementsNew, ContactLensCartNew, LoginElementsNew, PaymentPageElementsNew, SunglassCartNew for the above fixes and add diagnostic logging
</commit_message>
<xml_diff>
--- a/TestData/AddToCartNew.xlsx
+++ b/TestData/AddToCartNew.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paresh automation\Workspace\Titan-Mobile-Automation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1982741-E365-43DE-ACD0-62FFEBFD1A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C93CA1EB-6AC4-44B7-922F-7C55E806E847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -31,15 +31,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="34">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -131,14 +128,23 @@
     <t>DEFAULT_USER</t>
   </si>
   <si>
-    <t>M8022GY3V</t>
+    <t>Other UPI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC1241UFM2MBKGYV </t>
+  </si>
+  <si>
+    <t>TC1241UFM2MBKGYV </t>
+  </si>
+  <si>
+    <t>CJFAWD86</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -218,6 +224,18 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0F1D2A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0F1D2A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -240,7 +258,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -258,6 +276,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -573,22 +595,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B1BECAA-E7C3-4729-9704-A408DC33D20C}">
-  <dimension ref="A1:K42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K41"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="17.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -623,156 +645,154 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="5"/>
-      <c r="C2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="7"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="4"/>
       <c r="I2" s="6"/>
-      <c r="J2" t="s">
-        <v>26</v>
-      </c>
-      <c r="K2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J2" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C3" s="5"/>
       <c r="J3" s="12"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
       <c r="D4" s="7"/>
-      <c r="E4" s="5"/>
+      <c r="E4" s="13"/>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
       <c r="H4" s="4"/>
       <c r="I4" s="6"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="7"/>
-      <c r="E5" s="5"/>
+      <c r="E5" s="13"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
       <c r="H5" s="4"/>
       <c r="I5" s="6"/>
       <c r="J5" s="11"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="5"/>
+      <c r="E6" s="13"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="4"/>
       <c r="I6" s="6"/>
       <c r="J6" s="12"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I14" s="8"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I13" s="8"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I14" s="9"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="D15" s="8"/>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D16" s="8"/>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="D16" s="9"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D18" s="9"/>
+    <row r="18" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D18" s="10"/>
       <c r="I18" s="9"/>
     </row>
-    <row r="19" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D19" s="10"/>
-      <c r="I19" s="9"/>
-    </row>
-    <row r="20" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D20" s="9"/>
-      <c r="I20" s="10"/>
-    </row>
-    <row r="21" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D21" s="10"/>
-    </row>
-    <row r="22" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D19" s="9"/>
+      <c r="I19" s="10"/>
+    </row>
+    <row r="20" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D20" s="10"/>
+    </row>
+    <row r="21" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="I21" s="9"/>
+    </row>
+    <row r="22" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D22" s="8"/>
       <c r="I22" s="9"/>
     </row>
-    <row r="23" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D23" s="8"/>
       <c r="I23" s="9"/>
     </row>
-    <row r="24" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D24" s="8"/>
+    <row r="24" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D24" s="9"/>
       <c r="I24" s="9"/>
     </row>
-    <row r="25" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D25" s="9"/>
+    <row r="25" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D25" s="10"/>
       <c r="I25" s="9"/>
     </row>
-    <row r="26" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D26" s="10"/>
-      <c r="I26" s="9"/>
-    </row>
-    <row r="27" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D27" s="9"/>
-      <c r="I27" s="10"/>
-    </row>
-    <row r="28" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D28" s="10"/>
-    </row>
-    <row r="29" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="I29" s="8"/>
-    </row>
-    <row r="30" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D26" s="9"/>
+      <c r="I26" s="10"/>
+    </row>
+    <row r="27" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D27" s="10"/>
+    </row>
+    <row r="28" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="I28" s="8"/>
+    </row>
+    <row r="29" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="I29" s="9"/>
+    </row>
+    <row r="30" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="G30" s="10"/>
       <c r="I30" s="9"/>
     </row>
-    <row r="31" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="G31" s="10"/>
+    <row r="31" spans="4:9" x14ac:dyDescent="0.3">
       <c r="I31" s="9"/>
     </row>
-    <row r="32" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="I32" s="9"/>
-    </row>
-    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I33" s="10"/>
-    </row>
-    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I34" s="9"/>
-    </row>
-    <row r="35" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I35" s="10"/>
-    </row>
-    <row r="37" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="I32" s="10"/>
+    </row>
+    <row r="33" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I33" s="9"/>
+    </row>
+    <row r="34" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I34" s="10"/>
+    </row>
+    <row r="36" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I36" s="9"/>
+    </row>
+    <row r="37" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I37" s="9"/>
     </row>
-    <row r="38" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I38" s="9"/>
     </row>
-    <row r="39" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I39" s="9"/>
     </row>
-    <row r="40" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I40" s="9"/>
     </row>
-    <row r="41" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I41" s="9"/>
-    </row>
-    <row r="42" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I42" s="10"/>
+    <row r="41" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I41" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -783,12 +803,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02CAD0B7-4C47-44E3-ACD2-2B082261F449}">
   <dimension ref="A1:J51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="32.5703125" customWidth="1"/>
+    <col min="9" max="9" width="32.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -817,7 +837,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -846,12 +866,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>8</v>
       </c>
@@ -874,7 +894,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -903,7 +923,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>8</v>
       </c>
@@ -926,37 +946,42 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C13" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="H14" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="H15" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="H16" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H17" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H18" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>0</v>
       </c>
@@ -988,7 +1013,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>1</v>
       </c>
@@ -1006,7 +1031,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>2</v>
       </c>
@@ -1017,7 +1042,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>3</v>
       </c>
@@ -1049,7 +1074,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>4</v>
       </c>
@@ -1081,7 +1106,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>5</v>
       </c>
@@ -1120,10 +1145,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D340067D-92C5-4A87-863D-4C9C26FE9C40}">
-  <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O22"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="15" max="15" width="21.109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1155,7 +1183,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1173,7 +1201,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1184,7 +1212,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1215,8 +1243,11 @@
       <c r="J4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="O4" s="14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1248,7 +1279,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1280,7 +1311,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1294,7 +1325,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>3</v>
       </c>
@@ -1329,7 +1360,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>4</v>
       </c>
@@ -1364,7 +1395,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>5</v>
       </c>
@@ -1397,6 +1428,131 @@
       </c>
       <c r="K14" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>1</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J19" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>3</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>4</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>5</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update AddToCartNew test data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestData/AddToCartNew.xlsx
+++ b/TestData/AddToCartNew.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Titan-Mobile-Automation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paresh automation\Workspace\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C93CA1EB-6AC4-44B7-922F-7C55E806E847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{290B7590-7AB5-4E10-AF85-89480D413624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="39">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -138,13 +141,28 @@
   </si>
   <si>
     <t>CJFAWD86</t>
+  </si>
+  <si>
+    <t>SDS039BR3V </t>
+  </si>
+  <si>
+    <t>CJFAWD87</t>
+  </si>
+  <si>
+    <t>CJFAWD88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RxM253GY8PV </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FT1541UFP2MBRCGV </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,10 +249,16 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="9"/>
       <color rgb="FF0F1D2A"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -277,9 +301,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -596,21 +618,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B1BECAA-E7C3-4729-9704-A408DC33D20C}">
   <dimension ref="A1:K41"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.44140625" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" customWidth="1"/>
-    <col min="8" max="8" width="23.6640625" customWidth="1"/>
-    <col min="9" max="9" width="20.6640625" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -645,156 +667,222 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="C2" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="7"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="4"/>
       <c r="I2" s="6"/>
-      <c r="J2" s="11" t="s">
+      <c r="J2" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="5"/>
+      <c r="H4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="5"/>
+      <c r="H5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C3" s="5"/>
-      <c r="J3" s="12"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="6"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="11"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="5"/>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>37</v>
+      </c>
       <c r="G6" s="5"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="12"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I13" s="8"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I14" s="9"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D15" s="8"/>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D16" s="9"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D18" s="10"/>
       <c r="I18" s="9"/>
     </row>
-    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D19" s="9"/>
       <c r="I19" s="10"/>
     </row>
-    <row r="20" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D20" s="10"/>
     </row>
-    <row r="21" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I21" s="9"/>
     </row>
-    <row r="22" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D22" s="8"/>
       <c r="I22" s="9"/>
     </row>
-    <row r="23" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D23" s="8"/>
       <c r="I23" s="9"/>
     </row>
-    <row r="24" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D24" s="9"/>
       <c r="I24" s="9"/>
     </row>
-    <row r="25" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D25" s="10"/>
       <c r="I25" s="9"/>
     </row>
-    <row r="26" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D26" s="9"/>
       <c r="I26" s="10"/>
     </row>
-    <row r="27" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D27" s="10"/>
     </row>
-    <row r="28" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I28" s="8"/>
     </row>
-    <row r="29" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I29" s="9"/>
     </row>
-    <row r="30" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="4:9" x14ac:dyDescent="0.25">
       <c r="G30" s="10"/>
       <c r="I30" s="9"/>
     </row>
-    <row r="31" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I31" s="9"/>
     </row>
-    <row r="32" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I32" s="10"/>
     </row>
-    <row r="33" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I33" s="9"/>
     </row>
-    <row r="34" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I34" s="10"/>
     </row>
-    <row r="36" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I36" s="9"/>
     </row>
-    <row r="37" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I37" s="9"/>
     </row>
-    <row r="38" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I38" s="9"/>
     </row>
-    <row r="39" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I39" s="9"/>
     </row>
-    <row r="40" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I40" s="9"/>
     </row>
-    <row r="41" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I41" s="10"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -803,12 +891,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02CAD0B7-4C47-44E3-ACD2-2B082261F449}">
   <dimension ref="A1:J51"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="9" max="9" width="32.5546875" customWidth="1"/>
+    <col min="9" max="9" width="32.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -837,7 +925,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -866,12 +954,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>8</v>
       </c>
@@ -894,7 +982,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -923,12 +1011,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B11" s="5" t="s">
+    <row r="11" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="C11" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>16</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>18</v>
@@ -946,42 +1031,42 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C13" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H14" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H15" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H16" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H17" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H18" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>0</v>
       </c>
@@ -1013,7 +1098,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>1</v>
       </c>
@@ -1031,7 +1116,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2</v>
       </c>
@@ -1042,7 +1127,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>3</v>
       </c>
@@ -1074,7 +1159,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>4</v>
       </c>
@@ -1106,7 +1191,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>5</v>
       </c>
@@ -1140,18 +1225,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D340067D-92C5-4A87-863D-4C9C26FE9C40}">
   <dimension ref="A1:O22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="15" max="15" width="21.109375" customWidth="1"/>
+    <col min="15" max="15" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1183,7 +1269,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1201,7 +1287,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1212,7 +1298,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1243,11 +1329,11 @@
       <c r="J4" t="s">
         <v>22</v>
       </c>
-      <c r="O4" s="14" t="s">
+      <c r="O4" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1279,7 +1365,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1311,12 +1397,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>8</v>
+      <c r="C11" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="J11" s="12" t="s">
         <v>26</v>
@@ -1325,18 +1411,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>3</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>8</v>
+      <c r="C12" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>18</v>
@@ -1360,18 +1446,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>4</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>8</v>
+      <c r="C13" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>18</v>
@@ -1395,18 +1481,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>8</v>
+      <c r="C14" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>18</v>
@@ -1430,13 +1516,13 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>1</v>
       </c>
       <c r="B18" s="5"/>
-      <c r="C18" s="5" t="s">
-        <v>8</v>
+      <c r="C18" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="5"/>
@@ -1448,26 +1534,26 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>8</v>
+      <c r="C19" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="J19" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>8</v>
+      <c r="C20" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>16</v>
@@ -1476,13 +1562,13 @@
         <v>32</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>21</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="I20" s="6" t="s">
         <v>15</v>
@@ -1491,15 +1577,15 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>4</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>8</v>
+      <c r="C21" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>16</v>
@@ -1508,13 +1594,13 @@
         <v>32</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>21</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="I21" s="6" t="s">
         <v>15</v>
@@ -1523,15 +1609,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>5</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>8</v>
+      <c r="C22" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>16</v>
@@ -1540,13 +1626,13 @@
         <v>32</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>21</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="I22" s="6" t="s">
         <v>15</v>
@@ -1556,6 +1642,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix search suggestion and back-to-search flakiness in new-UI cart flow
- searchProduct: only use a displayed SUGGESTIONS node (a hidden leftover
  node was matched first and timed out), click that node, and fail with
  the SKU name plus a screenshot when no suggestion appears.
- backToSearch: detect Cart/PDP/Search/Home by unique markers and step
  back until Home, instead of treating any ImageView as the PDP (which
  tapped the Related Products card on the search screen).
- PurchaseDataReader: strip non-breaking spaces from SKUs.
- Update AddToCartNew test data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestData/AddToCartNew.xlsx
+++ b/TestData/AddToCartNew.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paresh automation\Workspace\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{290B7590-7AB5-4E10-AF85-89480D413624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D6064A-69BC-4F42-AB18-08F60E7BABE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="39">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -715,7 +715,9 @@
       <c r="F4" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="5"/>
+      <c r="G4" s="5" t="s">
+        <v>21</v>
+      </c>
       <c r="H4" s="4" t="s">
         <v>38</v>
       </c>
@@ -737,7 +739,7 @@
         <v>34</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>32</v>
@@ -745,7 +747,9 @@
       <c r="F5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G5" s="5"/>
+      <c r="G5" s="5" t="s">
+        <v>21</v>
+      </c>
       <c r="H5" s="4" t="s">
         <v>38</v>
       </c>
@@ -767,7 +771,7 @@
         <v>34</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>32</v>
@@ -775,7 +779,9 @@
       <c r="F6" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="5"/>
+      <c r="G6" s="5" t="s">
+        <v>21</v>
+      </c>
       <c r="H6" s="4" t="s">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Fix back-to-Home hang, Reading Glass power selection and wallet payment flow
- backToSearch: re-apply the 500ms implicit wait after each step, since
  click() restores the global 30s wait and stalled the screen detection;
  log screen trail and diagnostics on failure
- Reading Glass: pick +2.25 when selectable, else first in-stock power
  (out-of-stock powers are not clickable and the item was never added)
- Wallet/COD payment: confirm directly or continue via Razorpay, then
  verify "Order Confirmed."
- Update AddToCartNew test data

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestData/AddToCartNew.xlsx
+++ b/TestData/AddToCartNew.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paresh automation\Workspace\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D6064A-69BC-4F42-AB18-08F60E7BABE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE77BDF1-0386-410A-BFEC-979091C34397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
+    <workbookView xWindow="4965" yWindow="4125" windowWidth="14490" windowHeight="6795" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="39">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -617,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B1BECAA-E7C3-4729-9704-A408DC33D20C}">
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
@@ -668,37 +668,72 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5"/>
+      <c r="A2">
+        <v>3</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>31</v>
+      </c>
       <c r="C2" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="7"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="12" t="s">
-        <v>27</v>
+      <c r="D2" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="12" t="s">
-        <v>26</v>
+      <c r="D3" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>31</v>
@@ -724,138 +759,80 @@
       <c r="I4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="J4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>25</v>
       </c>
     </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I11" s="8"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I12" s="9"/>
+    </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="I13" s="9"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D14" s="9"/>
       <c r="I14" s="9"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D15" s="8"/>
+      <c r="D15" s="9"/>
       <c r="I15" s="9"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D16" s="9"/>
+      <c r="D16" s="10"/>
       <c r="I16" s="9"/>
     </row>
     <row r="17" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D17" s="9"/>
-      <c r="I17" s="9"/>
+      <c r="I17" s="10"/>
     </row>
     <row r="18" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D18" s="10"/>
-      <c r="I18" s="9"/>
     </row>
     <row r="19" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D19" s="9"/>
-      <c r="I19" s="10"/>
+      <c r="I19" s="9"/>
     </row>
     <row r="20" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D20" s="10"/>
+      <c r="D20" s="8"/>
+      <c r="I20" s="9"/>
     </row>
     <row r="21" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D21" s="8"/>
       <c r="I21" s="9"/>
     </row>
     <row r="22" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D22" s="8"/>
+      <c r="D22" s="9"/>
       <c r="I22" s="9"/>
     </row>
     <row r="23" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D23" s="8"/>
+      <c r="D23" s="10"/>
       <c r="I23" s="9"/>
     </row>
     <row r="24" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D24" s="9"/>
-      <c r="I24" s="9"/>
+      <c r="I24" s="10"/>
     </row>
     <row r="25" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D25" s="10"/>
-      <c r="I25" s="9"/>
     </row>
     <row r="26" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D26" s="9"/>
-      <c r="I26" s="10"/>
+      <c r="I26" s="8"/>
     </row>
     <row r="27" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D27" s="10"/>
+      <c r="I27" s="9"/>
     </row>
     <row r="28" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="I28" s="8"/>
+      <c r="G28" s="10"/>
+      <c r="I28" s="9"/>
     </row>
     <row r="29" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I29" s="9"/>
     </row>
     <row r="30" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="G30" s="10"/>
-      <c r="I30" s="9"/>
+      <c r="I30" s="10"/>
     </row>
     <row r="31" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I31" s="9"/>
@@ -863,11 +840,11 @@
     <row r="32" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I32" s="10"/>
     </row>
-    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I33" s="9"/>
-    </row>
     <row r="34" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I34" s="10"/>
+      <c r="I34" s="9"/>
+    </row>
+    <row r="35" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I35" s="9"/>
     </row>
     <row r="36" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I36" s="9"/>
@@ -879,13 +856,7 @@
       <c r="I38" s="9"/>
     </row>
     <row r="39" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I39" s="9"/>
-    </row>
-    <row r="40" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I40" s="9"/>
-    </row>
-    <row r="41" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I41" s="10"/>
+      <c r="I39" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>

</xml_diff>

<commit_message>
Fix out-of-stock popup check and remove-icon locator for out-of-stock rows
- proceedToCheckout: replace isDisplayed() on the "Remove all from cart"
  element with a non-throwing isElementPresent() check, since calling
  isDisplayed() on an absent element throws NoSuchElementException instead
  of returning false (this was failing every run where no out-of-stock
  popup appeared)
- RemoveProductsFromCartPAge: extend REMOVE_ICON_LOCATOR to also match
  out-of-stock rows' differently-styled "Remove" icon, and retarget
  removeButton to the ImageView variant confirmed via Appium Inspector
- Update AddToCartNew test data
</commit_message>
<xml_diff>
--- a/TestData/AddToCartNew.xlsx
+++ b/TestData/AddToCartNew.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paresh automation\Workspace\Titan-Mobile-Automation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE77BDF1-0386-410A-BFEC-979091C34397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA475B5-A01C-4F34-B185-AF992CCB6E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4965" yWindow="4125" windowWidth="14490" windowHeight="6795" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -31,15 +31,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="39">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -617,22 +614,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B1BECAA-E7C3-4729-9704-A408DC33D20C}">
-  <dimension ref="A1:K39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K41"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="17.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -667,73 +664,38 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>3</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>31</v>
-      </c>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5"/>
       <c r="C2" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D2" s="7"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>4</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J3" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>31</v>
@@ -759,104 +721,168 @@
       <c r="I4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I11" s="8"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D13" s="8"/>
-      <c r="I13" s="9"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D14" s="9"/>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I13" s="8"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="I14" s="9"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D15" s="9"/>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="D15" s="8"/>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D16" s="10"/>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="D16" s="9"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D17" s="9"/>
-      <c r="I17" s="10"/>
-    </row>
-    <row r="18" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="I17" s="9"/>
+    </row>
+    <row r="18" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D18" s="10"/>
-    </row>
-    <row r="19" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="I19" s="9"/>
-    </row>
-    <row r="20" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D20" s="8"/>
-      <c r="I20" s="9"/>
-    </row>
-    <row r="21" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D21" s="8"/>
+      <c r="I18" s="9"/>
+    </row>
+    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D19" s="9"/>
+      <c r="I19" s="10"/>
+    </row>
+    <row r="20" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D20" s="10"/>
+    </row>
+    <row r="21" spans="4:9" x14ac:dyDescent="0.3">
       <c r="I21" s="9"/>
     </row>
-    <row r="22" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D22" s="9"/>
+    <row r="22" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D22" s="8"/>
       <c r="I22" s="9"/>
     </row>
-    <row r="23" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="D23" s="10"/>
+    <row r="23" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D23" s="8"/>
       <c r="I23" s="9"/>
     </row>
-    <row r="24" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D24" s="9"/>
-      <c r="I24" s="10"/>
-    </row>
-    <row r="25" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="I24" s="9"/>
+    </row>
+    <row r="25" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D25" s="10"/>
-    </row>
-    <row r="26" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="I26" s="8"/>
-    </row>
-    <row r="27" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="I27" s="9"/>
-    </row>
-    <row r="28" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="G28" s="10"/>
-      <c r="I28" s="9"/>
-    </row>
-    <row r="29" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="I25" s="9"/>
+    </row>
+    <row r="26" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D26" s="9"/>
+      <c r="I26" s="10"/>
+    </row>
+    <row r="27" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D27" s="10"/>
+    </row>
+    <row r="28" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="I28" s="8"/>
+    </row>
+    <row r="29" spans="4:9" x14ac:dyDescent="0.3">
       <c r="I29" s="9"/>
     </row>
-    <row r="30" spans="4:9" x14ac:dyDescent="0.25">
-      <c r="I30" s="10"/>
-    </row>
-    <row r="31" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="G30" s="10"/>
+      <c r="I30" s="9"/>
+    </row>
+    <row r="31" spans="4:9" x14ac:dyDescent="0.3">
       <c r="I31" s="9"/>
     </row>
-    <row r="32" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:9" x14ac:dyDescent="0.3">
       <c r="I32" s="10"/>
     </row>
-    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I34" s="9"/>
-    </row>
-    <row r="35" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I35" s="9"/>
-    </row>
-    <row r="36" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I33" s="9"/>
+    </row>
+    <row r="34" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I34" s="10"/>
+    </row>
+    <row r="36" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I36" s="9"/>
     </row>
-    <row r="37" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I37" s="9"/>
     </row>
-    <row r="38" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I38" s="9"/>
     </row>
-    <row r="39" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I39" s="10"/>
+    <row r="39" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I39" s="9"/>
+    </row>
+    <row r="40" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I40" s="9"/>
+    </row>
+    <row r="41" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I41" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>
@@ -868,12 +894,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02CAD0B7-4C47-44E3-ACD2-2B082261F449}">
   <dimension ref="A1:J51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="32.5703125" customWidth="1"/>
+    <col min="9" max="9" width="32.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -902,7 +928,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -931,12 +957,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>8</v>
       </c>
@@ -959,7 +985,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -988,7 +1014,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="C11" s="5" t="s">
         <v>8</v>
       </c>
@@ -1008,42 +1034,42 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C13" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="H14" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="H15" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="H16" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H17" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H18" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>0</v>
       </c>
@@ -1075,7 +1101,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>1</v>
       </c>
@@ -1093,7 +1119,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>2</v>
       </c>
@@ -1104,7 +1130,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>3</v>
       </c>
@@ -1136,7 +1162,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>4</v>
       </c>
@@ -1168,7 +1194,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>5</v>
       </c>
@@ -1209,12 +1235,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D340067D-92C5-4A87-863D-4C9C26FE9C40}">
   <dimension ref="A1:O22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="15" max="15" width="21.140625" customWidth="1"/>
+    <col min="15" max="15" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1246,7 +1272,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1264,7 +1290,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1275,7 +1301,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1310,7 +1336,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1342,7 +1368,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1374,7 +1400,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1388,7 +1414,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>3</v>
       </c>
@@ -1423,7 +1449,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>4</v>
       </c>
@@ -1458,7 +1484,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>5</v>
       </c>
@@ -1493,7 +1519,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>1</v>
       </c>
@@ -1511,7 +1537,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2</v>
       </c>
@@ -1522,7 +1548,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1554,7 +1580,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>4</v>
       </c>
@@ -1586,7 +1612,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Fix BrowserStack purchase flow on Galaxy S24
- Pin Appium 3.5.2 and auto-grant permissions on BrowserStack
- Point BrowserStack at the Titan Eyewear build and default to browserstack mode
- Scroll contact lens power rows and Reading Glass power chips clear of the sticky Add to cart bar
- Accept negative Reading Glass powers as well as positive
- Scroll to the Titan Wallet section before selecting it
- Wait up to 90s for order confirmation on Other UPI
- Update AddToCartNew test data

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestData/AddToCartNew.xlsx
+++ b/TestData/AddToCartNew.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Titan-Mobile-Automation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paresh automation\Workspace\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA475B5-A01C-4F34-B185-AF992CCB6E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE4B4B0-FBB3-4B7D-BF0C-C474D52F29D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
+    <workbookView xWindow="6000" yWindow="1620" windowWidth="14490" windowHeight="6795" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -30,6 +30,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -615,21 +618,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B1BECAA-E7C3-4729-9704-A408DC33D20C}">
   <dimension ref="A1:K41"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.44140625" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" customWidth="1"/>
-    <col min="8" max="8" width="23.6640625" customWidth="1"/>
-    <col min="9" max="9" width="20.6640625" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -664,7 +667,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -682,7 +685,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -693,7 +696,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -725,7 +728,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -757,7 +760,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -789,99 +792,99 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I13" s="8"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I14" s="9"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D15" s="8"/>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D16" s="9"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D18" s="10"/>
       <c r="I18" s="9"/>
     </row>
-    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D19" s="9"/>
       <c r="I19" s="10"/>
     </row>
-    <row r="20" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D20" s="10"/>
     </row>
-    <row r="21" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I21" s="9"/>
     </row>
-    <row r="22" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D22" s="8"/>
       <c r="I22" s="9"/>
     </row>
-    <row r="23" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D23" s="8"/>
       <c r="I23" s="9"/>
     </row>
-    <row r="24" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D24" s="9"/>
       <c r="I24" s="9"/>
     </row>
-    <row r="25" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D25" s="10"/>
       <c r="I25" s="9"/>
     </row>
-    <row r="26" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D26" s="9"/>
       <c r="I26" s="10"/>
     </row>
-    <row r="27" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D27" s="10"/>
     </row>
-    <row r="28" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I28" s="8"/>
     </row>
-    <row r="29" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I29" s="9"/>
     </row>
-    <row r="30" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="4:9" x14ac:dyDescent="0.25">
       <c r="G30" s="10"/>
       <c r="I30" s="9"/>
     </row>
-    <row r="31" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I31" s="9"/>
     </row>
-    <row r="32" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I32" s="10"/>
     </row>
-    <row r="33" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I33" s="9"/>
     </row>
-    <row r="34" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I34" s="10"/>
     </row>
-    <row r="36" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I36" s="9"/>
     </row>
-    <row r="37" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I37" s="9"/>
     </row>
-    <row r="38" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I38" s="9"/>
     </row>
-    <row r="39" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I39" s="9"/>
     </row>
-    <row r="40" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I40" s="9"/>
     </row>
-    <row r="41" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I41" s="10"/>
     </row>
   </sheetData>
@@ -894,12 +897,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02CAD0B7-4C47-44E3-ACD2-2B082261F449}">
   <dimension ref="A1:J51"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="9" max="9" width="32.5546875" customWidth="1"/>
+    <col min="9" max="9" width="32.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -928,7 +931,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -957,12 +960,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>8</v>
       </c>
@@ -985,7 +988,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -1014,7 +1017,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="C11" s="5" t="s">
         <v>8</v>
       </c>
@@ -1034,42 +1037,42 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C13" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H14" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H15" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H16" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H17" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H18" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>0</v>
       </c>
@@ -1101,7 +1104,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>1</v>
       </c>
@@ -1119,7 +1122,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2</v>
       </c>
@@ -1130,7 +1133,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>3</v>
       </c>
@@ -1162,7 +1165,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>4</v>
       </c>
@@ -1194,7 +1197,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>5</v>
       </c>
@@ -1235,12 +1238,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D340067D-92C5-4A87-863D-4C9C26FE9C40}">
   <dimension ref="A1:O22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="15" max="15" width="21.109375" customWidth="1"/>
+    <col min="15" max="15" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1272,7 +1275,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1290,7 +1293,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1301,7 +1304,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1336,7 +1339,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1368,7 +1371,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1400,7 +1403,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1414,7 +1417,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>3</v>
       </c>
@@ -1449,7 +1452,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>4</v>
       </c>
@@ -1484,7 +1487,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5</v>
       </c>
@@ -1519,7 +1522,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>1</v>
       </c>
@@ -1537,7 +1540,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2</v>
       </c>
@@ -1548,7 +1551,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1580,7 +1583,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>4</v>
       </c>
@@ -1612,7 +1615,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>5</v>
       </c>

</xml_diff>